<commit_message>
reduced line power capacity to 1MW
</commit_message>
<xml_diff>
--- a/data/links.xlsx
+++ b/data/links.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Geteilte Ablagen\KEKS- Kores\Code\Pypsa proto\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Keks-repo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C1BFE8-2FD5-4640-91B0-1AF69A75EDE4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9702C24C-C146-4386-BC39-6702460EBCB9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -529,7 +529,7 @@
         <v>0.95</v>
       </c>
       <c r="G3" s="1">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="I3">
         <v>-1</v>
@@ -552,7 +552,7 @@
         <v>0.95</v>
       </c>
       <c r="G4" s="1">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="I4">
         <v>-1</v>
@@ -575,7 +575,7 @@
         <v>0.95</v>
       </c>
       <c r="G5" s="1">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="I5">
         <v>-1</v>

</xml_diff>